<commit_message>
Fix member visibility and audit loading
</commit_message>
<xml_diff>
--- a/test-kit/Beplan全系统测试数据与用例_V2.0.xlsx
+++ b/test-kit/Beplan全系统测试数据与用例_V2.0.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试总览" sheetId="1" r:id="Rc331ae6ae4844d7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="账号与权限" sheetId="2" r:id="R8d316557c6564ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主数据" sheetId="3" r:id="Rb482f817b94e4e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合同流程" sheetId="4" r:id="Reee473c1bece477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全系统用例" sheetId="5" r:id="Rf4a0c77f8849462b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件清单" sheetId="6" r:id="R6dc9ae4656a84bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="权限矩阵" sheetId="7" r:id="R6cb8a5dd4c7948d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺陷记录" sheetId="8" r:id="R828bb1b8e54d479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试总结" sheetId="9" r:id="R8507e9db14ad430d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试总览" sheetId="1" r:id="R758aa10c1ab645df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="账号与权限" sheetId="2" r:id="Rf6d9ae2d7b9941df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主数据" sheetId="3" r:id="Rbdae1cae03934aa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合同流程" sheetId="4" r:id="Rcdbeaf2031544929"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全系统用例" sheetId="5" r:id="R71177ab164e24caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件清单" sheetId="6" r:id="R92cd0a727f4546f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="权限矩阵" sheetId="7" r:id="R68ae023e7e75466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺陷记录" sheetId="8" r:id="Rac03aaaf9e404c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试总结" sheetId="9" r:id="R02e6202754b74054"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,7 +472,7 @@
         <x:v>测试环境</x:v>
       </x:c>
       <x:c r="B4" s="22" t="str">
-        <x:v>Vercel + Supabase 托管云</x:v>
+        <x:v>GitHub Pages + Supabase 托管云</x:v>
       </x:c>
       <x:c r="C4" s="22" t="str">
         <x:v>同事可从其他电脑访问；业务数据仍需邮箱登录和组织授权</x:v>
@@ -483,7 +483,7 @@
         <x:v>测试网址</x:v>
       </x:c>
       <x:c r="B5" s="23" t="str">
-        <x:v>https://beplan-caseops-uat.vercel.app</x:v>
+        <x:v>https://chenguanyu-cgy.github.io</x:v>
       </x:c>
       <x:c r="C5" s="23" t="str">
         <x:v>公开网页入口，不公开业务数据</x:v>

</xml_diff>